<commit_message>
prompt abalation matching error fixed
</commit_message>
<xml_diff>
--- a/Analysis/Listwise_Direct/listwise_summary.xlsx
+++ b/Analysis/Listwise_Direct/listwise_summary.xlsx
@@ -489,22 +489,22 @@
         <v>5</v>
       </c>
       <c r="D2" t="n">
-        <v>0.109652014016209</v>
+        <v>0.1152136752136752</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3733333333333334</v>
+        <v>0.3712820512820513</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6871794871794871</v>
+        <v>0.686153846153846</v>
       </c>
       <c r="G2" t="n">
-        <v>0.03218719945979839</v>
+        <v>0.03080719405420529</v>
       </c>
       <c r="H2" t="n">
-        <v>0.03064075742828647</v>
+        <v>0.02654805970368161</v>
       </c>
       <c r="I2" t="n">
-        <v>0.01776462366737311</v>
+        <v>0.02217615211327145</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -528,22 +528,22 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>0.03030472671019283</v>
+        <v>0.03247863247863249</v>
       </c>
       <c r="E3" t="n">
-        <v>0.3466666666666666</v>
+        <v>0.3405128205128205</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6707692307692308</v>
+        <v>0.6656410256410257</v>
       </c>
       <c r="G3" t="n">
-        <v>0.02842412706088412</v>
+        <v>0.02558398213178763</v>
       </c>
       <c r="H3" t="n">
-        <v>0.023667652839414</v>
+        <v>0.02193769193457173</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0281818085416084</v>
+        <v>0.03148734652924873</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -567,22 +567,22 @@
         <v>5</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1405058426363512</v>
+        <v>0.1343589743589743</v>
       </c>
       <c r="E4" t="n">
-        <v>0.3774358974358974</v>
+        <v>0.3682051282051282</v>
       </c>
       <c r="F4" t="n">
-        <v>0.7035897435897436</v>
+        <v>0.6984615384615385</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0404458750330653</v>
+        <v>0.04040846308948344</v>
       </c>
       <c r="H4" t="n">
-        <v>0.02775870482610124</v>
+        <v>0.02771129453560267</v>
       </c>
       <c r="I4" t="n">
-        <v>0.01111768378906607</v>
+        <v>0.01169410692409372</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -606,22 +606,22 @@
         <v>5</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.000668236688872274</v>
+        <v>0.005470085470085467</v>
       </c>
       <c r="E5" t="n">
-        <v>0.3046153846153846</v>
+        <v>0.3076923076923077</v>
       </c>
       <c r="F5" t="n">
         <v>0.6646153846153846</v>
       </c>
       <c r="G5" t="n">
-        <v>0.03360466434391415</v>
+        <v>0.03734172286061715</v>
       </c>
       <c r="H5" t="n">
-        <v>0.02252911039639877</v>
+        <v>0.02459400781186011</v>
       </c>
       <c r="I5" t="n">
-        <v>0.02629924390760632</v>
+        <v>0.02475388386901984</v>
       </c>
       <c r="J5" t="n">
         <v>2.2</v>
@@ -645,22 +645,22 @@
         <v>5</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2415798001157747</v>
+        <v>0.2464957264957265</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4</v>
+        <v>0.3969230769230769</v>
       </c>
       <c r="F6" t="n">
-        <v>0.7158974358974359</v>
+        <v>0.7107692307692307</v>
       </c>
       <c r="G6" t="n">
-        <v>0.01779940052935179</v>
+        <v>0.01983937250250141</v>
       </c>
       <c r="H6" t="n">
-        <v>0.01025641025641025</v>
+        <v>0.01337272288246699</v>
       </c>
       <c r="I6" t="n">
-        <v>0.01939248246275799</v>
+        <v>0.01939248246275797</v>
       </c>
       <c r="J6" t="n">
         <v>4</v>
@@ -684,22 +684,22 @@
         <v>5</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1253094358866817</v>
+        <v>0.1247863247863248</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3948717948717949</v>
+        <v>0.3907692307692308</v>
       </c>
       <c r="F7" t="n">
-        <v>0.7343589743589745</v>
+        <v>0.7292307692307693</v>
       </c>
       <c r="G7" t="n">
-        <v>0.02693207654323542</v>
+        <v>0.03095858166884587</v>
       </c>
       <c r="H7" t="n">
-        <v>0.019527623348369</v>
+        <v>0.02841414395322066</v>
       </c>
       <c r="I7" t="n">
-        <v>0.02674544576493395</v>
+        <v>0.02443308564014687</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -723,19 +723,19 @@
         <v>5</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2168262677883441</v>
+        <v>0.2225641025641026</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3928205128205128</v>
+        <v>0.3938461538461538</v>
       </c>
       <c r="F8" t="n">
-        <v>0.72</v>
+        <v>0.7148717948717949</v>
       </c>
       <c r="G8" t="n">
-        <v>0.005921541222457692</v>
+        <v>0.004586806107691885</v>
       </c>
       <c r="H8" t="n">
-        <v>0.004586806107691882</v>
+        <v>0.007606357422662212</v>
       </c>
       <c r="I8" t="n">
         <v>0.00458680610769186</v>
@@ -762,19 +762,19 @@
         <v>5</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1719208082230964</v>
+        <v>0.1788034188034188</v>
       </c>
       <c r="E9" t="n">
-        <v>0.398974358974359</v>
+        <v>0.3979487179487179</v>
       </c>
       <c r="F9" t="n">
-        <v>0.7076923076923076</v>
+        <v>0.7025641025641025</v>
       </c>
       <c r="G9" t="n">
-        <v>0.02015061933050946</v>
+        <v>0.01955005600751561</v>
       </c>
       <c r="H9" t="n">
-        <v>0.009864299518805809</v>
+        <v>0.007777308147745182</v>
       </c>
       <c r="I9" t="n">
         <v>0.009593993299420388</v>
@@ -894,13 +894,13 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>6547</v>
+        <v>6432.5</v>
       </c>
       <c r="F2" t="n">
-        <v>0.006642830321172535</v>
+        <v>0.007756040998386563</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2306698002350176</v>
+        <v>0.2274665225484898</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -908,10 +908,10 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="J2" t="n">
-        <v>0.1100328731097962</v>
+        <v>0.1086653517422748</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
         <v>195</v>
       </c>
       <c r="M2" t="n">
-        <v>0.06642830321172535</v>
+        <v>0.07756040998386562</v>
       </c>
       <c r="N2" t="b">
         <v>0</v>
@@ -950,24 +950,24 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>4033.5</v>
+        <v>4140.5</v>
       </c>
       <c r="F3" t="n">
-        <v>0.3404923254356699</v>
+        <v>0.2580738635743676</v>
       </c>
       <c r="G3" t="n">
-        <v>0.09471439793513635</v>
+        <v>0.1110991841992271</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>negligible</t>
+          <t>small</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="J3" t="n">
-        <v>0.0333990795529257</v>
+        <v>0.03936883629191321</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -1006,13 +1006,13 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>4072.5</v>
+        <v>4098.5</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1998125219603605</v>
+        <v>0.1742450814114346</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1256977243452125</v>
+        <v>0.1328678726330265</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -1020,10 +1020,10 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J4" t="n">
-        <v>0.0756870479947403</v>
+        <v>0.08226166995397764</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -1062,13 +1062,13 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>6430</v>
+        <v>6154</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0003436510434263112</v>
+        <v>0.001594593792054399</v>
       </c>
       <c r="G5" t="n">
-        <v>0.2986474694589878</v>
+        <v>0.2689474934663816</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1076,10 +1076,10 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="J5" t="n">
-        <v>0.1759894806048652</v>
+        <v>0.1578698224852071</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -1090,7 +1090,7 @@
         <v>195</v>
       </c>
       <c r="M5" t="n">
-        <v>0.004123812521115735</v>
+        <v>0.01754053171259839</v>
       </c>
       <c r="N5" t="b">
         <v>1</v>
@@ -1118,13 +1118,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>3343.5</v>
+        <v>3470</v>
       </c>
       <c r="F6" t="n">
-        <v>0.01200476243428086</v>
+        <v>0.03567589243964163</v>
       </c>
       <c r="G6" t="n">
-        <v>0.2495791718101223</v>
+        <v>0.2093871041239462</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -1132,10 +1132,10 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J6" t="n">
-        <v>0.042077580539119</v>
+        <v>0.0210913872452334</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -1146,7 +1146,7 @@
         <v>195</v>
       </c>
       <c r="M6" t="n">
-        <v>0.1080428619085277</v>
+        <v>0.285407139517133</v>
       </c>
       <c r="N6" t="b">
         <v>0</v>
@@ -1174,24 +1174,24 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>4947</v>
+        <v>4986</v>
       </c>
       <c r="F7" t="n">
-        <v>0.2760262657708746</v>
+        <v>0.3786051969174223</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1026664248140758</v>
+        <v>0.08328736900165472</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>negligible</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J7" t="n">
-        <v>0.1715713346482577</v>
+        <v>0.1603155818540434</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -1230,35 +1230,35 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>6237.5</v>
+        <v>5366</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0003975387181834663</v>
+        <v>0.0003444698156083182</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2978160531352021</v>
+        <v>0.3109912686183873</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>176</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.1566863905325444</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
           <t>small</t>
         </is>
       </c>
-      <c r="I8" t="n">
-        <v>188</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0.1622616699539776</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>small</t>
-        </is>
-      </c>
       <c r="L8" t="n">
         <v>195</v>
       </c>
       <c r="M8" t="n">
-        <v>0.004372925900018129</v>
+        <v>0.004133637787299818</v>
       </c>
       <c r="N8" t="b">
         <v>1</v>
@@ -1286,13 +1286,13 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>4849.5</v>
+        <v>4854.5</v>
       </c>
       <c r="F9" t="n">
-        <v>0.9738854704665069</v>
+        <v>0.9823097009619217</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.003186022610483042</v>
+        <v>-0.002158273381294964</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -1303,7 +1303,7 @@
         <v>139</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.05840894148586456</v>
+        <v>-0.06111768573307035</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1314,7 +1314,7 @@
         <v>195</v>
       </c>
       <c r="M9" t="n">
-        <v>0.9738854704665069</v>
+        <v>0.9823097009619217</v>
       </c>
       <c r="N9" t="b">
         <v>0</v>
@@ -1342,13 +1342,13 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>2710.5</v>
+        <v>2756.5</v>
       </c>
       <c r="F10" t="n">
-        <v>0.304094636271096</v>
+        <v>0.297625103158942</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.112039312039312</v>
+        <v>-0.1130952380952381</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -1356,10 +1356,10 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J10" t="n">
-        <v>0.08936226166995398</v>
+        <v>0.08704799474030243</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1398,24 +1398,24 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>3312</v>
+        <v>1033</v>
       </c>
       <c r="F11" t="n">
-        <v>0.05064201687520581</v>
+        <v>0.01710405730232087</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1976744186046512</v>
+        <v>0.312021312021312</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>128</v>
+        <v>77</v>
       </c>
       <c r="J11" t="n">
-        <v>0.02666666666666667</v>
+        <v>0.01914529914529915</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1426,7 +1426,7 @@
         <v>195</v>
       </c>
       <c r="M11" t="n">
-        <v>0.4051361350016465</v>
+        <v>0.1539365157208878</v>
       </c>
       <c r="N11" t="b">
         <v>0</v>
@@ -1454,13 +1454,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>434</v>
+        <v>443</v>
       </c>
       <c r="F12" t="n">
-        <v>0.6359018394386931</v>
+        <v>0.7157222010336191</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.0824524312896406</v>
+        <v>-0.06342494714587738</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1471,7 +1471,7 @@
         <v>43</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.01717291255752794</v>
+        <v>-0.01664694280078895</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>

</xml_diff>